<commit_message>
some file in auxiliary has been modified
</commit_message>
<xml_diff>
--- a/src/dibs_data/data/auxiliary/occupancy_schedules/occupancy_schedules_SIA2024.xlsx
+++ b/src/dibs_data/data/auxiliary/occupancy_schedules/occupancy_schedules_SIA2024.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6CA8B49-0D0D-4044-98C0-ADDB5D9CC8D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SIA2024" sheetId="2" r:id="rId1"/>
     <sheet name="Zuweisungen" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Zuweisungen!$A$1:$B$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Zuweisungen!$A$1:$B$109</definedName>
     <definedName name="Hotel">'SIA2024'!$B$3:$B$4</definedName>
     <definedName name="Industrie">'SIA2024'!$B$32:$B$34</definedName>
     <definedName name="Lager">'SIA2024'!$B$35</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="188">
   <si>
     <t>Sterne-Hotel</t>
   </si>
@@ -583,13 +584,22 @@
     <t>Gebäude für gewerbliche Produktion und Verarbeitung (z.B. Brauerei, Molkerei, Schlachthof)</t>
   </si>
   <si>
-    <t>WohnenMFH</t>
+    <t>Wohngebäude</t>
+  </si>
+  <si>
+    <t>Ein- und Zweifamilienhaus</t>
+  </si>
+  <si>
+    <t>Mehrfamilienhaus</t>
+  </si>
+  <si>
+    <t>Wohnen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -629,12 +639,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="13">
@@ -797,7 +813,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
@@ -842,6 +858,8 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -851,16 +869,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1142,23 +1160,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="45.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>158</v>
       </c>
@@ -1190,7 +1208,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -1206,15 +1224,15 @@
       <c r="E2" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
       <c r="J2" s="12" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -1224,17 +1242,17 @@
       <c r="C3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="28"/>
       <c r="J3" s="13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -1256,13 +1274,13 @@
       <c r="G4" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="H4" s="28"/>
-      <c r="I4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="31"/>
       <c r="J4" s="13" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -1278,15 +1296,15 @@
       <c r="E5" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="26"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="28"/>
       <c r="J5" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -1296,17 +1314,17 @@
       <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="28"/>
       <c r="J6" s="13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -1316,17 +1334,17 @@
       <c r="C7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="28"/>
       <c r="J7" s="13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -1336,17 +1354,17 @@
       <c r="C8" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="28"/>
       <c r="J8" s="13" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>8</v>
       </c>
@@ -1356,17 +1374,17 @@
       <c r="C9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="28"/>
       <c r="J9" s="13" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>9</v>
       </c>
@@ -1376,17 +1394,17 @@
       <c r="C10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="28"/>
       <c r="J10" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>10</v>
       </c>
@@ -1396,17 +1414,17 @@
       <c r="C11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="28"/>
+      <c r="D11" s="29"/>
       <c r="E11" s="30"/>
       <c r="F11" s="30"/>
       <c r="G11" s="30"/>
       <c r="H11" s="30"/>
-      <c r="I11" s="29"/>
+      <c r="I11" s="31"/>
       <c r="J11" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>11</v>
       </c>
@@ -1416,17 +1434,17 @@
       <c r="C12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="28"/>
       <c r="J12" s="13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>12</v>
       </c>
@@ -1436,17 +1454,17 @@
       <c r="C13" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="28"/>
       <c r="J13" s="13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>13</v>
       </c>
@@ -1456,17 +1474,17 @@
       <c r="C14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="28"/>
       <c r="J14" s="13" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>14</v>
       </c>
@@ -1476,17 +1494,17 @@
       <c r="C15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="28"/>
       <c r="J15" s="13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
         <v>15</v>
       </c>
@@ -1496,17 +1514,17 @@
       <c r="C16" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="28"/>
       <c r="J16" s="13" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
         <v>16</v>
       </c>
@@ -1516,17 +1534,17 @@
       <c r="C17" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="28"/>
       <c r="J17" s="13" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>17</v>
       </c>
@@ -1536,17 +1554,17 @@
       <c r="C18" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="28"/>
       <c r="J18" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -1556,17 +1574,17 @@
       <c r="C19" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
       <c r="J19" s="13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
         <v>19</v>
       </c>
@@ -1576,17 +1594,17 @@
       <c r="C20" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="28"/>
+      <c r="D20" s="29"/>
       <c r="E20" s="30"/>
       <c r="F20" s="30"/>
       <c r="G20" s="30"/>
       <c r="H20" s="30"/>
-      <c r="I20" s="29"/>
+      <c r="I20" s="31"/>
       <c r="J20" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7">
         <v>20</v>
       </c>
@@ -1602,15 +1620,15 @@
       <c r="E21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="28"/>
+      <c r="F21" s="29"/>
       <c r="G21" s="30"/>
       <c r="H21" s="30"/>
-      <c r="I21" s="29"/>
+      <c r="I21" s="31"/>
       <c r="J21" s="13" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
         <v>21</v>
       </c>
@@ -1626,15 +1644,15 @@
       <c r="E22" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F22" s="24"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="28"/>
       <c r="J22" s="13" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>22</v>
       </c>
@@ -1644,17 +1662,17 @@
       <c r="C23" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="28"/>
+      <c r="D23" s="29"/>
       <c r="E23" s="30"/>
       <c r="F23" s="30"/>
       <c r="G23" s="30"/>
       <c r="H23" s="30"/>
-      <c r="I23" s="29"/>
+      <c r="I23" s="31"/>
       <c r="J23" s="13" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
         <v>23</v>
       </c>
@@ -1664,17 +1682,17 @@
       <c r="C24" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="28"/>
       <c r="J24" s="13" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
         <v>24</v>
       </c>
@@ -1684,17 +1702,17 @@
       <c r="C25" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="28"/>
       <c r="J25" s="13" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
         <v>25</v>
       </c>
@@ -1704,100 +1722,90 @@
       <c r="C26" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="28"/>
       <c r="J26" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C32" s="2"/>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" s="2"/>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38" s="2"/>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40" s="2"/>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" s="2"/>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" s="2"/>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" s="2"/>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47" s="2"/>
     </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" s="2"/>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C49" s="2"/>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C50" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="D24:I24"/>
-    <mergeCell ref="D26:I26"/>
-    <mergeCell ref="D25:I25"/>
-    <mergeCell ref="D15:I15"/>
-    <mergeCell ref="D20:I20"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="D18:I18"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="D23:I23"/>
     <mergeCell ref="D14:I14"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="D17:I17"/>
@@ -1813,6 +1821,16 @@
     <mergeCell ref="D9:I9"/>
     <mergeCell ref="D10:I10"/>
     <mergeCell ref="D12:I12"/>
+    <mergeCell ref="D24:I24"/>
+    <mergeCell ref="D26:I26"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D15:I15"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="D23:I23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1820,16 +1838,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C98"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C112"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="84.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.5546875" customWidth="1"/>
-    <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="84.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.5703125" customWidth="1"/>
+    <col min="3" max="3" width="47.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>153</v>
       </c>
@@ -1840,1071 +1858,1177 @@
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="24"/>
+      <c r="C2" s="25"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>66</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>66</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>66</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>66</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>73</v>
+        <v>156</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B15" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
+    <row r="16" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B30" s="24"/>
+      <c r="C30" s="25"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B42" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
         <v>2</v>
       </c>
       <c r="B47" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B52" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C52" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="15" t="s">
+    <row r="53" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B48" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B52" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B53" s="24"/>
+      <c r="C53" s="25"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>8</v>
+        <v>118</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B63" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B66" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B68" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C63" s="6" t="s">
+      <c r="C69" s="6" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="15" t="s">
+    <row r="70" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="B64" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B65" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B66" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B67" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B68" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B69" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B70" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="24"/>
+      <c r="C70" s="25"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
         <v>125</v>
       </c>
       <c r="B71" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B74" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B75" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B76" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B77" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B78" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C71" s="6" t="s">
+      <c r="C78" s="6" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="15" t="s">
+    <row r="79" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="B72" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B73" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B74" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B75" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B76" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B77" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B78" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B79" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B79" s="24"/>
+      <c r="C79" s="25"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
         <v>131</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>139</v>
+        <v>183</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
         <v>131</v>
       </c>
       <c r="B81" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B83" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B84" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B85" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B86" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B87" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B88" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B89" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="C81" s="6" t="s">
+      <c r="C89" s="6" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A82" s="14" t="s">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B90" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C82" s="6" t="s">
+      <c r="C90" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" s="14" t="s">
+    <row r="91" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B83" s="14" t="s">
+      <c r="B91" s="24"/>
+      <c r="C91" s="25"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B92" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="C83" s="6" t="s">
+      <c r="C92" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" s="14" t="s">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B84" s="14" t="s">
+      <c r="B93" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="C84" s="6" t="s">
+      <c r="C93" s="6" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" s="14" t="s">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B85" s="14" t="s">
+      <c r="B94" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B86" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B87" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A88" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B88" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B89" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C89" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A90" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B90" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="C90" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B91" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A92" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B92" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A93" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B93" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A94" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B94" s="16" t="s">
-        <v>18</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B95" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B96" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B97" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B98" s="24"/>
+      <c r="C98" s="25"/>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B99" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B100" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B101" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B102" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B103" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B104" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B95" s="14" t="s">
+      <c r="B105" s="24"/>
+      <c r="C105" s="25"/>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B106" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C95" s="6" t="s">
+      <c r="C106" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" s="14" t="s">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B96" s="14" t="s">
+      <c r="B107" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="C96" s="6" t="s">
+      <c r="C107" s="6" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A97" s="14" t="s">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B97" s="14" t="s">
+      <c r="B108" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="C97" s="6" t="s">
+      <c r="C108" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="14" t="s">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B98" s="14" t="s">
+      <c r="B109" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="C98" s="6" t="s">
+      <c r="C109" s="6" t="s">
         <v>180</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="B110" s="24"/>
+      <c r="C110" s="25"/>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B111" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B112" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2914,11 +3038,11 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
             <xm:f>'SIA2024'!$J$2:$J$26</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C98</xm:sqref>
+          <xm:sqref>C2:C112</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>